<commit_message>
Redesenho da UI, gráfico de professores necessários e ajustes de RH
Adiciona cálculo de profissionais necessários (professor+monitor) por dia,
com visualização no gráfico da aba Professores, rodapé por semana no
Calendário, tarja nos cards e tooltip nos botões de módulo. Reestrutura
abas (remove Visão Geral/Grade Detalhada/Por Semana), adiciona filtro por
módulo, redesenha cores da UI e ajusta exportação CSV/XLSX por semana.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CFP 3 AGENTES.xlsx
+++ b/CFP 3 AGENTES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcelfelipeprocopiodemoura/Documents/PROJETOS CLAUDE/GRADE PRELIMINAR 3 CFP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEFDCB20-D784-2C42-AA55-B22164809C7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2509014-E8FB-BA4A-9700-6D8F41DEFEFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-3060" yWindow="-21100" windowWidth="38400" windowHeight="19640" xr2:uid="{A5D0A619-F59C-1444-BB10-0F263888FD23}"/>
+    <workbookView xWindow="16140" yWindow="-21100" windowWidth="19200" windowHeight="19480" xr2:uid="{A5D0A619-F59C-1444-BB10-0F263888FD23}"/>
   </bookViews>
   <sheets>
     <sheet name="DESCRIÇÃO" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="62">
   <si>
     <t>PLANTÃO</t>
   </si>
@@ -220,6 +220,12 @@
   </si>
   <si>
     <t>EXCLUIR FAZER A IPJ E INCLUIR SLIDE</t>
+  </si>
+  <si>
+    <t>RECURSOS HUMANOS PROFESSOR</t>
+  </si>
+  <si>
+    <t>RECURSOS HUMANOS MONITOR</t>
   </si>
 </sst>
 </file>
@@ -261,7 +267,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -269,15 +275,41 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -612,248 +644,384 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FA8892D-A7FF-CF4B-8050-C22E4E48951D}">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" customWidth="1"/>
-    <col min="4" max="4" width="22.6640625" customWidth="1"/>
-    <col min="5" max="5" width="19.33203125" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="4" max="4" width="13.1640625" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" customWidth="1"/>
+    <col min="6" max="6" width="22.6640625" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" spans="1:7" s="8" customFormat="1" ht="73" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="C1" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" s="8" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="C2" s="3">
+        <v>8</v>
+      </c>
+      <c r="D2" s="3">
+        <v>4</v>
+      </c>
+      <c r="E2" s="3">
+        <v>2</v>
+      </c>
+      <c r="F2" t="s">
         <v>37</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="2">
-        <v>2</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="C5" s="4">
+        <v>8</v>
+      </c>
+      <c r="D5" s="4">
+        <v>5</v>
+      </c>
+      <c r="E5" s="4">
+        <v>2</v>
+      </c>
+      <c r="F5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="2">
-        <v>4</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="C6" s="4">
+        <v>12</v>
+      </c>
+      <c r="D6" s="4">
+        <v>1</v>
+      </c>
+      <c r="E6" s="4">
+        <v>4</v>
+      </c>
+      <c r="F6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+      <c r="C7" s="4">
         <v>10</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="D7" s="4">
+        <v>8</v>
+      </c>
+      <c r="E7" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
+      <c r="C8" s="4">
+        <v>13</v>
+      </c>
+      <c r="D8" s="4">
+        <v>0</v>
+      </c>
+      <c r="E8" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
+      <c r="C9" s="4">
+        <v>11</v>
+      </c>
+      <c r="D9" s="4">
+        <v>8</v>
+      </c>
+      <c r="E9" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
+      <c r="C10" s="4">
+        <v>10</v>
+      </c>
+      <c r="D10" s="4">
+        <v>0</v>
+      </c>
+      <c r="E10" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
+      <c r="C11" s="4">
+        <v>5</v>
+      </c>
+      <c r="D11" s="4">
+        <v>0</v>
+      </c>
+      <c r="E11" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A12" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="3">
-        <v>2</v>
-      </c>
-      <c r="D13" t="s">
+      <c r="C13" s="5">
+        <v>11</v>
+      </c>
+      <c r="D13" s="5">
+        <v>1</v>
+      </c>
+      <c r="E13" s="5">
+        <v>2</v>
+      </c>
+      <c r="F13" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="3" t="s">
+      <c r="C14" s="5">
+        <v>2</v>
+      </c>
+      <c r="D14" s="5">
+        <v>4</v>
+      </c>
+      <c r="E14" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="3" t="s">
+      <c r="C15" s="5">
+        <v>16</v>
+      </c>
+      <c r="D15" s="5">
+        <v>14</v>
+      </c>
+      <c r="E15" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="3" t="s">
+      <c r="C16" s="5">
+        <v>2</v>
+      </c>
+      <c r="D16" s="5">
+        <v>4</v>
+      </c>
+      <c r="E16" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
+      <c r="C17" s="5">
+        <v>2</v>
+      </c>
+      <c r="D17" s="5">
+        <v>6</v>
+      </c>
+      <c r="E17" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C18" s="3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="3" t="s">
+      <c r="C18" s="5">
+        <v>10</v>
+      </c>
+      <c r="D18" s="5">
+        <v>8</v>
+      </c>
+      <c r="E18" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C19" s="3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="3" t="s">
+      <c r="C19" s="5">
+        <v>3</v>
+      </c>
+      <c r="D19" s="5">
+        <v>8</v>
+      </c>
+      <c r="E19" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C20" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" s="3" t="s">
+      <c r="C20" s="5">
+        <v>6</v>
+      </c>
+      <c r="D20" s="5">
+        <v>4</v>
+      </c>
+      <c r="E20" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C21" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="C22">
-        <f>SUM(C2:C21)</f>
+      <c r="C21" s="5">
+        <v>1</v>
+      </c>
+      <c r="D21" s="5">
+        <v>2</v>
+      </c>
+      <c r="E21" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E22">
+        <f>SUM(E2:E21)</f>
         <v>50</v>
       </c>
     </row>

</xml_diff>